<commit_message>
Deployed  with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/courses/apply_py/data/xls_data.xlsx
+++ b/courses/apply_py/data/xls_data.xlsx
@@ -442,42 +442,42 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.0551789006252525</v>
+        <v>0.4376514728863113</v>
       </c>
       <c r="B2" t="n">
-        <v>0.9033339210880966</v>
+        <v>0.2258175749476771</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.5854362060453604</v>
+        <v>0.7745765040869125</v>
       </c>
       <c r="B3" t="n">
-        <v>0.3483943248681471</v>
+        <v>0.0360997536951448</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.89970017095815</v>
+        <v>0.4704178211696445</v>
       </c>
       <c r="B4" t="n">
-        <v>0.3595605964154288</v>
+        <v>0.4031302016491758</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.9396820579673808</v>
+        <v>0.4201729486806285</v>
       </c>
       <c r="B5" t="n">
-        <v>0.4488847590015233</v>
+        <v>0.8647192768269525</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.2283378236664572</v>
+        <v>0.8651066069762412</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0300379403747007</v>
+        <v>0.9547802363307512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>